<commit_message>
Add 'Group' column to the machine status table and update header management
</commit_message>
<xml_diff>
--- a/Mappa_nodi.xlsx
+++ b/Mappa_nodi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camozzicloud-my.sharepoint.com/personal/mpasseri_fonderiemoragavardo_it/Documents/Documenti/VSCode/EnergyMeters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="523" documentId="11_CBF82CE5D29271A855494D68F3BC070891C844B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF921028-FB44-42E8-92CC-B0698E0E22AB}"/>
+  <xr:revisionPtr revIDLastSave="525" documentId="11_CBF82CE5D29271A855494D68F3BC070891C844B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F3F9D3A-ED2E-4921-9183-FDDE101ACAEC}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="213" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="213" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -2504,10 +2504,11 @@
       </c>
       <c r="G51" s="6"/>
       <c r="H51" s="27" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="I51" s="28">
-        <v>10000</v>
+        <f>400/0.333</f>
+        <v>1201.2012012012012</v>
       </c>
       <c r="J51" s="27" t="s">
         <v>175</v>

</xml_diff>

<commit_message>
Update binary files Mappa_nodi.xlsx and Utenze_main.xlsx
</commit_message>
<xml_diff>
--- a/Mappa_nodi.xlsx
+++ b/Mappa_nodi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camozzicloud-my.sharepoint.com/personal/mpasseri_fonderiemoragavardo_it/Documents/Documenti/VSCode/EnergyMeters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="525" documentId="11_CBF82CE5D29271A855494D68F3BC070891C844B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F3F9D3A-ED2E-4921-9183-FDDE101ACAEC}"/>
+  <xr:revisionPtr revIDLastSave="527" documentId="11_CBF82CE5D29271A855494D68F3BC070891C844B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8111D4E-4EA1-4D98-BC36-8AEBE4F3C1CF}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="213" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30135" yWindow="2220" windowWidth="21600" windowHeight="11175" tabRatio="213" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Mappa_nodi.xlsx with latest data revisions
</commit_message>
<xml_diff>
--- a/Mappa_nodi.xlsx
+++ b/Mappa_nodi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camozzicloud-my.sharepoint.com/personal/mpasseri_fonderiemoragavardo_it/Documents/Documenti/VSCode/EnergyMeters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="527" documentId="11_CBF82CE5D29271A855494D68F3BC070891C844B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8111D4E-4EA1-4D98-BC36-8AEBE4F3C1CF}"/>
+  <xr:revisionPtr revIDLastSave="531" documentId="11_CBF82CE5D29271A855494D68F3BC070891C844B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0348118-84DB-44A8-8DD2-2D8AB6EE1251}"/>
   <bookViews>
-    <workbookView xWindow="30135" yWindow="2220" windowWidth="21600" windowHeight="11175" tabRatio="213" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="213" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="182">
   <si>
     <t>Cabina</t>
   </si>
@@ -96,9 +96,6 @@
     <t>175A   3Fx95  pompe raffreddamento forni</t>
   </si>
   <si>
-    <t>utenza sbagliata e modulo scollegato</t>
-  </si>
-  <si>
     <t>7</t>
   </si>
   <si>
@@ -510,9 +507,6 @@
     <t>QI-KCT-35-300/333</t>
   </si>
   <si>
-    <t>Manca</t>
-  </si>
-  <si>
     <t>Rogowski QI-R0G-400-A</t>
   </si>
   <si>
@@ -586,6 +580,9 @@
   </si>
   <si>
     <t>OK</t>
+  </si>
+  <si>
+    <t>Nuova centrale oleodinamica pistone H1 - Hydroven</t>
   </si>
 </sst>
 </file>
@@ -596,7 +593,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.000_-;\-* #,##0.000_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -620,13 +617,6 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -728,7 +718,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -798,22 +788,19 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -825,7 +812,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -847,10 +834,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1167,22 +1150,22 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>149</v>
-      </c>
       <c r="F1" s="17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -1196,19 +1179,19 @@
         <v>4</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F2" s="4">
         <v>35</v>
       </c>
       <c r="G2" s="21"/>
-      <c r="H2" s="31" t="s">
-        <v>158</v>
-      </c>
-      <c r="I2" s="26">
+      <c r="H2" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="I2" s="25">
         <v>10000</v>
       </c>
       <c r="J2" s="6"/>
@@ -1231,10 +1214,10 @@
         <v>35</v>
       </c>
       <c r="G3" s="21"/>
-      <c r="H3" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="I3" s="26">
+      <c r="H3" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="I3" s="25">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
@@ -1254,18 +1237,18 @@
         <v>10</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F4" s="4">
         <v>35</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="H4" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="H4" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="I4" s="26">
+      <c r="I4" s="25">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
@@ -1285,18 +1268,18 @@
         <v>13</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F5" s="4">
         <v>35</v>
       </c>
-      <c r="G5" s="33" t="s">
+      <c r="G5" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="H5" s="30" t="s">
         <v>150</v>
       </c>
-      <c r="H5" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="I5" s="26">
+      <c r="I5" s="25">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
@@ -1320,16 +1303,16 @@
         <v>35</v>
       </c>
       <c r="G6" s="21"/>
-      <c r="H6" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="I6" s="26">
+      <c r="H6" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="I6" s="25">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
       <c r="J6" s="6"/>
     </row>
-    <row r="7" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="22" t="s">
         <v>3</v>
       </c>
@@ -1340,17 +1323,19 @@
         <v>18</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>19</v>
+        <v>181</v>
       </c>
       <c r="E7" s="23"/>
       <c r="F7" s="4">
         <v>35</v>
       </c>
       <c r="G7" s="21"/>
-      <c r="H7" s="25" t="s">
-        <v>157</v>
-      </c>
-      <c r="I7" s="26"/>
+      <c r="H7" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="I7" s="25">
+        <v>900.9</v>
+      </c>
       <c r="J7" s="6"/>
     </row>
     <row r="8" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -1358,23 +1343,23 @@
         <v>3</v>
       </c>
       <c r="B8" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="D8" s="23" t="s">
         <v>21</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>22</v>
       </c>
       <c r="E8" s="23"/>
       <c r="F8" s="4">
         <v>35</v>
       </c>
       <c r="G8" s="21"/>
-      <c r="H8" s="31" t="s">
-        <v>154</v>
-      </c>
-      <c r="I8" s="26">
+      <c r="H8" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="I8" s="25">
         <v>10000</v>
       </c>
       <c r="J8" s="6"/>
@@ -1384,23 +1369,23 @@
         <v>3</v>
       </c>
       <c r="B9" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="D9" s="23" t="s">
         <v>24</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>25</v>
       </c>
       <c r="E9" s="23"/>
       <c r="F9" s="4">
         <v>35</v>
       </c>
       <c r="G9" s="21"/>
-      <c r="H9" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="I9" s="26">
+      <c r="H9" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="I9" s="25">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
@@ -1411,23 +1396,23 @@
         <v>3</v>
       </c>
       <c r="B10" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="D10" s="23" t="s">
         <v>27</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>28</v>
       </c>
       <c r="E10" s="23"/>
       <c r="F10" s="4">
         <v>35</v>
       </c>
       <c r="G10" s="21"/>
-      <c r="H10" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="I10" s="26">
+      <c r="H10" s="30" t="s">
+        <v>155</v>
+      </c>
+      <c r="I10" s="25">
         <v>900.9</v>
       </c>
       <c r="J10" s="6"/>
@@ -1437,23 +1422,23 @@
         <v>3</v>
       </c>
       <c r="B11" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="D11" s="23" t="s">
         <v>30</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>31</v>
       </c>
       <c r="E11" s="23"/>
       <c r="F11" s="4">
         <v>35</v>
       </c>
       <c r="G11" s="21"/>
-      <c r="H11" s="31" t="s">
-        <v>151</v>
-      </c>
-      <c r="I11" s="26">
+      <c r="H11" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="I11" s="25">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
@@ -1464,23 +1449,23 @@
         <v>3</v>
       </c>
       <c r="B12" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="D12" s="23" t="s">
         <v>33</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>34</v>
       </c>
       <c r="E12" s="23"/>
       <c r="F12" s="4">
         <v>35</v>
       </c>
       <c r="G12" s="21"/>
-      <c r="H12" s="31" t="s">
-        <v>154</v>
-      </c>
-      <c r="I12" s="26">
+      <c r="H12" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="I12" s="25">
         <v>10000</v>
       </c>
       <c r="J12" s="6"/>
@@ -1490,22 +1475,22 @@
         <v>3</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C13" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="23" t="s">
-        <v>37</v>
-      </c>
       <c r="F13" s="4">
         <v>35</v>
       </c>
       <c r="G13" s="21"/>
-      <c r="H13" s="31" t="s">
-        <v>154</v>
-      </c>
-      <c r="I13" s="26">
+      <c r="H13" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="I13" s="25">
         <v>10000</v>
       </c>
       <c r="J13" s="6"/>
@@ -1515,25 +1500,25 @@
         <v>3</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14" s="20" t="s">
         <v>4</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F14" s="4">
         <v>35</v>
       </c>
       <c r="G14" s="21"/>
-      <c r="H14" s="31" t="s">
-        <v>158</v>
-      </c>
-      <c r="I14" s="26">
+      <c r="H14" s="30" t="s">
+        <v>156</v>
+      </c>
+      <c r="I14" s="25">
         <v>10000</v>
       </c>
       <c r="J14" s="6"/>
@@ -1543,28 +1528,28 @@
         <v>3</v>
       </c>
       <c r="B15" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="D15" s="16" t="s">
         <v>40</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>41</v>
       </c>
       <c r="E15" s="11"/>
       <c r="F15" s="4">
         <v>35</v>
       </c>
       <c r="G15" s="6"/>
-      <c r="H15" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I15" s="30">
+      <c r="H15" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I15" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J15" s="27" t="s">
-        <v>175</v>
+      <c r="J15" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -1572,28 +1557,28 @@
         <v>3</v>
       </c>
       <c r="B16" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="E16" s="11"/>
       <c r="F16" s="4">
         <v>35</v>
       </c>
       <c r="G16" s="6"/>
-      <c r="H16" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I16" s="30">
+      <c r="H16" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I16" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J16" s="27" t="s">
-        <v>175</v>
+      <c r="J16" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -1601,28 +1586,28 @@
         <v>3</v>
       </c>
       <c r="B17" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="D17" s="10" t="s">
         <v>46</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>47</v>
       </c>
       <c r="E17" s="11"/>
       <c r="F17" s="4">
         <v>35</v>
       </c>
       <c r="G17" s="6"/>
-      <c r="H17" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I17" s="30">
+      <c r="H17" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I17" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J17" s="27" t="s">
-        <v>175</v>
+      <c r="J17" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -1630,28 +1615,28 @@
         <v>3</v>
       </c>
       <c r="B18" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>49</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>50</v>
       </c>
       <c r="E18" s="11"/>
       <c r="F18" s="4">
         <v>35</v>
       </c>
       <c r="G18" s="6"/>
-      <c r="H18" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I18" s="30">
+      <c r="H18" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I18" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J18" s="27" t="s">
-        <v>175</v>
+      <c r="J18" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -1659,28 +1644,28 @@
         <v>3</v>
       </c>
       <c r="B19" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="D19" s="10" t="s">
         <v>52</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="E19" s="11"/>
       <c r="F19" s="4">
         <v>35</v>
       </c>
       <c r="G19" s="6"/>
-      <c r="H19" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I19" s="30">
+      <c r="H19" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I19" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J19" s="27" t="s">
-        <v>175</v>
+      <c r="J19" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -1688,50 +1673,50 @@
         <v>3</v>
       </c>
       <c r="B20" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="D20" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D20" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" s="35"/>
+      <c r="E20" s="34"/>
       <c r="F20" s="4">
         <v>35</v>
       </c>
       <c r="G20" s="6"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="27"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="26"/>
     </row>
     <row r="21" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>3</v>
       </c>
       <c r="B21" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="D21" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>59</v>
       </c>
       <c r="E21" s="11"/>
       <c r="F21" s="4">
         <v>35</v>
       </c>
       <c r="G21" s="6"/>
-      <c r="H21" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I21" s="30">
+      <c r="H21" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I21" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J21" s="27" t="s">
-        <v>175</v>
+      <c r="J21" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="33.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1739,28 +1724,28 @@
         <v>3</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="D22" s="10" t="s">
         <v>61</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>62</v>
       </c>
       <c r="E22" s="11"/>
       <c r="F22" s="4">
         <v>35</v>
       </c>
       <c r="G22" s="6"/>
-      <c r="H22" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I22" s="30">
+      <c r="H22" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I22" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J22" s="27" t="s">
-        <v>175</v>
+      <c r="J22" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -1768,28 +1753,28 @@
         <v>3</v>
       </c>
       <c r="B23" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="D23" s="10" t="s">
         <v>64</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>65</v>
       </c>
       <c r="E23" s="11"/>
       <c r="F23" s="4">
         <v>35</v>
       </c>
       <c r="G23" s="6"/>
-      <c r="H23" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I23" s="30">
+      <c r="H23" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I23" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J23" s="27" t="s">
-        <v>175</v>
+      <c r="J23" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -1797,27 +1782,27 @@
         <v>3</v>
       </c>
       <c r="B24" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="D24" s="10" t="s">
         <v>67</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>68</v>
       </c>
       <c r="E24" s="11"/>
       <c r="F24" s="4">
         <v>35</v>
       </c>
       <c r="G24" s="6"/>
-      <c r="H24" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="I24" s="28">
+      <c r="H24" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="I24" s="27">
         <v>10000</v>
       </c>
-      <c r="J24" s="27" t="s">
-        <v>175</v>
+      <c r="J24" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="87" x14ac:dyDescent="0.35">
@@ -1825,13 +1810,13 @@
         <v>3</v>
       </c>
       <c r="B25" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="D25" s="10" t="s">
         <v>70</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>71</v>
       </c>
       <c r="E25" s="11"/>
       <c r="F25" s="4">
@@ -1847,13 +1832,13 @@
         <v>3</v>
       </c>
       <c r="B26" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="D26" s="10" t="s">
         <v>73</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>74</v>
       </c>
       <c r="E26" s="11"/>
       <c r="F26" s="4">
@@ -1868,13 +1853,13 @@
         <v>3</v>
       </c>
       <c r="B27" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C27" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="C27" s="10" t="s">
-        <v>76</v>
-      </c>
       <c r="D27" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E27" s="11"/>
       <c r="F27" s="4">
@@ -1890,27 +1875,27 @@
         <v>3</v>
       </c>
       <c r="B28" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="D28" s="10" t="s">
         <v>78</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>79</v>
       </c>
       <c r="E28" s="11"/>
       <c r="F28" s="4">
         <v>35</v>
       </c>
       <c r="G28" s="6"/>
-      <c r="H28" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="I28" s="28">
+      <c r="H28" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="I28" s="27">
         <v>10000</v>
       </c>
-      <c r="J28" s="27" t="s">
-        <v>175</v>
+      <c r="J28" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -1924,17 +1909,17 @@
         <v>4</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F29" s="4">
         <v>35</v>
       </c>
       <c r="G29" s="7"/>
       <c r="H29" s="7" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="I29" s="13">
         <v>10000</v>
@@ -1949,18 +1934,18 @@
         <v>5</v>
       </c>
       <c r="C30" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D30" s="10" t="s">
         <v>80</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>81</v>
       </c>
       <c r="E30" s="11"/>
       <c r="F30" s="4">
         <v>35</v>
       </c>
       <c r="G30" s="6"/>
-      <c r="H30" s="31" t="s">
-        <v>169</v>
+      <c r="H30" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="I30" s="13">
         <f>400/0.333</f>
@@ -1976,18 +1961,18 @@
         <v>8</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E31" s="11"/>
       <c r="F31" s="4">
         <v>35</v>
       </c>
       <c r="G31" s="6"/>
-      <c r="H31" s="31" t="s">
-        <v>169</v>
+      <c r="H31" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="I31" s="13">
         <f>400/0.333</f>
@@ -2003,20 +1988,20 @@
         <v>11</v>
       </c>
       <c r="C32" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D32" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="D32" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="E32" s="32" t="s">
-        <v>172</v>
+      <c r="E32" s="31" t="s">
+        <v>170</v>
       </c>
       <c r="F32" s="4">
         <v>35</v>
       </c>
       <c r="G32" s="6"/>
-      <c r="H32" s="31" t="s">
-        <v>169</v>
+      <c r="H32" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="I32" s="13">
         <f>400/0.333</f>
@@ -2032,18 +2017,18 @@
         <v>14</v>
       </c>
       <c r="C33" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>85</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>86</v>
       </c>
       <c r="E33" s="11"/>
       <c r="F33" s="4">
         <v>35</v>
       </c>
       <c r="G33" s="6"/>
-      <c r="H33" s="31" t="s">
-        <v>154</v>
+      <c r="H33" s="30" t="s">
+        <v>153</v>
       </c>
       <c r="I33" s="13">
         <v>10000</v>
@@ -2058,18 +2043,18 @@
         <v>17</v>
       </c>
       <c r="C34" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>87</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>88</v>
       </c>
       <c r="E34" s="11"/>
       <c r="F34" s="4">
         <v>35</v>
       </c>
       <c r="G34" s="6"/>
-      <c r="H34" s="31" t="s">
-        <v>169</v>
+      <c r="H34" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="I34" s="13">
         <f>400/0.333</f>
@@ -2082,21 +2067,21 @@
         <v>5</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C35" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35" s="10" t="s">
         <v>89</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>90</v>
       </c>
       <c r="E35" s="11"/>
       <c r="F35" s="4">
         <v>35</v>
       </c>
       <c r="G35" s="6"/>
-      <c r="H35" s="31" t="s">
-        <v>154</v>
+      <c r="H35" s="30" t="s">
+        <v>153</v>
       </c>
       <c r="I35" s="13">
         <v>10000</v>
@@ -2108,21 +2093,21 @@
         <v>5</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C36" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36" s="10" t="s">
         <v>91</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>92</v>
       </c>
       <c r="E36" s="11"/>
       <c r="F36" s="4">
         <v>35</v>
       </c>
       <c r="G36" s="6"/>
-      <c r="H36" s="31" t="s">
-        <v>169</v>
+      <c r="H36" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="I36" s="13">
         <f>400/0.333</f>
@@ -2135,21 +2120,21 @@
         <v>5</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C37" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D37" s="10" t="s">
         <v>93</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>94</v>
       </c>
       <c r="E37" s="11"/>
       <c r="F37" s="4">
         <v>35</v>
       </c>
       <c r="G37" s="6"/>
-      <c r="H37" s="31" t="s">
-        <v>169</v>
+      <c r="H37" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="I37" s="13">
         <f>400/0.333</f>
@@ -2162,21 +2147,21 @@
         <v>5</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C38" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D38" s="10" t="s">
         <v>95</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>96</v>
       </c>
       <c r="E38" s="11"/>
       <c r="F38" s="4">
         <v>35</v>
       </c>
       <c r="G38" s="6"/>
-      <c r="H38" s="31" t="s">
-        <v>169</v>
+      <c r="H38" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="I38" s="13">
         <f>400/0.333</f>
@@ -2189,28 +2174,28 @@
         <v>5</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C39" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D39" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>98</v>
       </c>
       <c r="E39" s="11"/>
       <c r="F39" s="4">
         <v>35</v>
       </c>
       <c r="G39" s="6"/>
-      <c r="H39" s="27" t="s">
-        <v>170</v>
-      </c>
-      <c r="I39" s="27">
+      <c r="H39" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="I39" s="26">
         <f>400/0.033</f>
         <v>12121.21212121212</v>
       </c>
-      <c r="J39" s="27" t="s">
-        <v>174</v>
+      <c r="J39" s="26" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -2218,21 +2203,21 @@
         <v>5</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C40" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D40" s="10" t="s">
         <v>99</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>100</v>
       </c>
       <c r="E40" s="11"/>
       <c r="F40" s="4">
         <v>35</v>
       </c>
       <c r="G40" s="6"/>
-      <c r="H40" s="31" t="s">
-        <v>156</v>
+      <c r="H40" s="30" t="s">
+        <v>155</v>
       </c>
       <c r="I40" s="13">
         <f>300/0.333</f>
@@ -2245,21 +2230,21 @@
         <v>5</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C41" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41" s="10" t="s">
         <v>101</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>102</v>
       </c>
       <c r="E41" s="11"/>
       <c r="F41" s="4">
         <v>35</v>
       </c>
       <c r="G41" s="6"/>
-      <c r="H41" s="31" t="s">
-        <v>169</v>
+      <c r="H41" s="30" t="s">
+        <v>167</v>
       </c>
       <c r="I41" s="13">
         <f>400/0.333</f>
@@ -2272,23 +2257,23 @@
         <v>5</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C42" s="12" t="s">
         <v>4</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E42" s="24" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F42" s="4">
         <v>35</v>
       </c>
       <c r="G42" s="6"/>
-      <c r="H42" s="31" t="s">
-        <v>158</v>
+      <c r="H42" s="30" t="s">
+        <v>156</v>
       </c>
       <c r="I42" s="13">
         <v>10000</v>
@@ -2300,13 +2285,13 @@
         <v>5</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C43" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D43" s="10" t="s">
         <v>104</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>105</v>
       </c>
       <c r="E43" s="11"/>
       <c r="F43" s="4">
@@ -2322,13 +2307,13 @@
         <v>5</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C44" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D44" s="10" t="s">
         <v>106</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>107</v>
       </c>
       <c r="E44" s="11"/>
       <c r="F44" s="4">
@@ -2344,21 +2329,21 @@
         <v>5</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C45" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D45" s="10" t="s">
         <v>108</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>109</v>
       </c>
       <c r="E45" s="11"/>
       <c r="F45" s="4">
         <v>35</v>
       </c>
       <c r="G45" s="6"/>
-      <c r="H45" s="31" t="s">
-        <v>154</v>
+      <c r="H45" s="30" t="s">
+        <v>153</v>
       </c>
       <c r="I45" s="13">
         <v>10000</v>
@@ -2370,13 +2355,13 @@
         <v>5</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C46" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="D46" s="10" t="s">
         <v>110</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>111</v>
       </c>
       <c r="E46" s="11"/>
       <c r="F46" s="4">
@@ -2392,21 +2377,21 @@
         <v>5</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C47" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="D47" s="10" t="s">
         <v>112</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>113</v>
       </c>
       <c r="E47" s="11"/>
       <c r="F47" s="4">
         <v>35</v>
       </c>
       <c r="G47" s="6"/>
-      <c r="H47" s="31" t="s">
-        <v>154</v>
+      <c r="H47" s="30" t="s">
+        <v>153</v>
       </c>
       <c r="I47" s="13">
         <v>10000</v>
@@ -2418,21 +2403,21 @@
         <v>5</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C48" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="D48" s="10" t="s">
         <v>114</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>115</v>
       </c>
       <c r="E48" s="11"/>
       <c r="F48" s="4">
         <v>35</v>
       </c>
       <c r="G48" s="6"/>
-      <c r="H48" s="31" t="s">
-        <v>171</v>
+      <c r="H48" s="30" t="s">
+        <v>169</v>
       </c>
       <c r="I48" s="13"/>
       <c r="J48" s="6"/>
@@ -2442,13 +2427,13 @@
         <v>5</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C49" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="D49" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>117</v>
       </c>
       <c r="E49" s="11"/>
       <c r="F49" s="4">
@@ -2470,10 +2455,10 @@
         <v>4</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E50" s="24" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F50" s="4">
         <v>35</v>
@@ -2491,27 +2476,27 @@
         <v>5</v>
       </c>
       <c r="C51" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="D51" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="D51" s="10" t="s">
-        <v>119</v>
-      </c>
       <c r="E51" s="24" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F51" s="4">
         <v>35</v>
       </c>
       <c r="G51" s="6"/>
-      <c r="H51" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="I51" s="28">
+      <c r="H51" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="I51" s="27">
         <f>400/0.333</f>
         <v>1201.2012012012012</v>
       </c>
-      <c r="J51" s="27" t="s">
-        <v>175</v>
+      <c r="J51" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -2522,23 +2507,23 @@
         <v>8</v>
       </c>
       <c r="C52" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D52" s="10" t="s">
         <v>120</v>
-      </c>
-      <c r="D52" s="10" t="s">
-        <v>121</v>
       </c>
       <c r="E52" s="11"/>
       <c r="F52" s="4">
         <v>35</v>
       </c>
-      <c r="H52" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="I52" s="28">
+      <c r="H52" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="I52" s="27">
         <v>10000</v>
       </c>
-      <c r="J52" s="27" t="s">
-        <v>175</v>
+      <c r="J52" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -2549,26 +2534,26 @@
         <v>11</v>
       </c>
       <c r="C53" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D53" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="D53" s="10" t="s">
-        <v>123</v>
-      </c>
       <c r="E53" s="24" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F53" s="4">
         <v>35</v>
       </c>
       <c r="G53" s="6"/>
-      <c r="H53" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="I53" s="28">
+      <c r="H53" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="I53" s="27">
         <v>10000</v>
       </c>
-      <c r="J53" s="27" t="s">
-        <v>175</v>
+      <c r="J53" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -2579,25 +2564,25 @@
         <v>14</v>
       </c>
       <c r="C54" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D54" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="E54" s="11"/>
       <c r="F54" s="4">
         <v>35</v>
       </c>
       <c r="G54" s="6"/>
-      <c r="H54" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I54" s="30">
+      <c r="H54" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I54" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J54" s="27" t="s">
-        <v>175</v>
+      <c r="J54" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -2608,13 +2593,13 @@
         <v>17</v>
       </c>
       <c r="C55" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="D55" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="D55" s="10" t="s">
-        <v>127</v>
-      </c>
       <c r="E55" s="11" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F55" s="4">
         <v>35</v>
@@ -2629,28 +2614,28 @@
         <v>8</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C56" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="D56" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="D56" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="E56" s="34"/>
+      <c r="E56" s="33"/>
       <c r="F56" s="4">
         <v>35</v>
       </c>
       <c r="G56" s="6"/>
-      <c r="H56" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I56" s="30">
+      <c r="H56" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I56" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J56" s="27" t="s">
-        <v>175</v>
+      <c r="J56" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -2658,28 +2643,28 @@
         <v>8</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C57" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="D57" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="D57" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="E57" s="11"/>
       <c r="F57" s="4">
         <v>35</v>
       </c>
       <c r="G57" s="6"/>
-      <c r="H57" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I57" s="30">
+      <c r="H57" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I57" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J57" s="27" t="s">
-        <v>175</v>
+      <c r="J57" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -2687,28 +2672,28 @@
         <v>8</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C58" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D58" s="10" t="s">
         <v>132</v>
-      </c>
-      <c r="D58" s="10" t="s">
-        <v>133</v>
       </c>
       <c r="E58" s="11"/>
       <c r="F58" s="4">
         <v>35</v>
       </c>
       <c r="G58" s="6"/>
-      <c r="H58" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I58" s="30">
+      <c r="H58" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I58" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J58" s="27" t="s">
-        <v>175</v>
+      <c r="J58" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -2716,28 +2701,28 @@
         <v>8</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C59" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D59" s="10" t="s">
         <v>134</v>
-      </c>
-      <c r="D59" s="10" t="s">
-        <v>135</v>
       </c>
       <c r="E59" s="11"/>
       <c r="F59" s="4">
         <v>35</v>
       </c>
       <c r="G59" s="6"/>
-      <c r="H59" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I59" s="30">
+      <c r="H59" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I59" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J59" s="27" t="s">
-        <v>175</v>
+      <c r="J59" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
@@ -2745,28 +2730,28 @@
         <v>8</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C60" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D60" s="10" t="s">
         <v>136</v>
-      </c>
-      <c r="D60" s="10" t="s">
-        <v>137</v>
       </c>
       <c r="E60" s="11"/>
       <c r="F60" s="4">
         <v>35</v>
       </c>
       <c r="G60" s="6"/>
-      <c r="H60" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="I60" s="28">
+      <c r="H60" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="I60" s="27">
         <f>400/0.333</f>
         <v>1201.2012012012012</v>
       </c>
-      <c r="J60" s="27" t="s">
-        <v>175</v>
+      <c r="J60" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -2774,28 +2759,28 @@
         <v>8</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C61" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E61" s="11"/>
       <c r="F61" s="4">
         <v>35</v>
       </c>
       <c r="G61" s="6"/>
-      <c r="H61" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="I61" s="30">
+      <c r="H61" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="I61" s="29">
         <f>200/0.333</f>
         <v>600.60060060060061</v>
       </c>
-      <c r="J61" s="27" t="s">
-        <v>175</v>
+      <c r="J61" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -2803,28 +2788,28 @@
         <v>8</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C62" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D62" s="10" t="s">
         <v>139</v>
-      </c>
-      <c r="D62" s="10" t="s">
-        <v>140</v>
       </c>
       <c r="E62" s="11"/>
       <c r="F62" s="4">
         <v>35</v>
       </c>
       <c r="G62" s="6"/>
-      <c r="H62" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="I62" s="28">
+      <c r="H62" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="I62" s="27">
         <f>400/0.333</f>
         <v>1201.2012012012012</v>
       </c>
-      <c r="J62" s="27" t="s">
-        <v>175</v>
+      <c r="J62" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="63" spans="1:10" ht="29" x14ac:dyDescent="0.35">
@@ -2832,27 +2817,27 @@
         <v>8</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C63" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D63" s="10" t="s">
         <v>141</v>
-      </c>
-      <c r="D63" s="10" t="s">
-        <v>142</v>
       </c>
       <c r="E63" s="11"/>
       <c r="F63" s="4">
         <v>35</v>
       </c>
       <c r="G63" s="6"/>
-      <c r="H63" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="I63" s="28">
+      <c r="H63" s="26" t="s">
+        <v>174</v>
+      </c>
+      <c r="I63" s="27">
         <v>10000</v>
       </c>
-      <c r="J63" s="27" t="s">
-        <v>175</v>
+      <c r="J63" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="58" x14ac:dyDescent="0.35">
@@ -2860,28 +2845,28 @@
         <v>8</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C64" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="D64" s="10" t="s">
         <v>143</v>
-      </c>
-      <c r="D64" s="10" t="s">
-        <v>144</v>
       </c>
       <c r="E64" s="11"/>
       <c r="F64" s="4">
         <v>35</v>
       </c>
       <c r="G64" s="6"/>
-      <c r="H64" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="I64" s="28">
+      <c r="H64" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="I64" s="27">
         <f>400/0.333</f>
         <v>1201.2012012012012</v>
       </c>
-      <c r="J64" s="27" t="s">
-        <v>175</v>
+      <c r="J64" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="65" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
@@ -2889,28 +2874,28 @@
         <v>8</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C65" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="D65" s="10" t="s">
         <v>145</v>
-      </c>
-      <c r="D65" s="10" t="s">
-        <v>146</v>
       </c>
       <c r="E65" s="11"/>
       <c r="F65" s="4">
         <v>35</v>
       </c>
       <c r="G65" s="6"/>
-      <c r="H65" s="27" t="s">
-        <v>169</v>
-      </c>
-      <c r="I65" s="28">
+      <c r="H65" s="26" t="s">
+        <v>167</v>
+      </c>
+      <c r="I65" s="27">
         <f>400/0.333</f>
         <v>1201.2012012012012</v>
       </c>
-      <c r="J65" s="27" t="s">
-        <v>175</v>
+      <c r="J65" s="26" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -2929,18 +2914,18 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.35">
@@ -2956,18 +2941,18 @@
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.35">
@@ -2983,7 +2968,7 @@
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D8" s="5">
         <v>2958</v>
@@ -3030,7 +3015,7 @@
         <v>16502</v>
       </c>
       <c r="D12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F12">
         <v>27.65</v>

</xml_diff>